<commit_message>
Fix env variable loading in notebook
</commit_message>
<xml_diff>
--- a/dashboard/Loan_Portfolio_Analytics_Report.xlsx
+++ b/dashboard/Loan_Portfolio_Analytics_Report.xlsx
@@ -490,16 +490,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>95</v>
+        <v>307</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>238424496.79</v>
+        <v>771035733.54</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2509731.55</v>
+        <v>2511517.05</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>47.5</v>
+        <v>51.17</v>
       </c>
     </row>
     <row r="3">
@@ -509,16 +509,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>140484792.83</v>
+        <v>379529118.75</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2809695.86</v>
+        <v>2710922.28</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>25</v>
+        <v>23.33</v>
       </c>
     </row>
     <row r="4">
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>46</v>
+        <v>130</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>122976071.41</v>
+        <v>340012006.07</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2673392.86</v>
+        <v>2615476.97</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>23</v>
+        <v>21.67</v>
       </c>
     </row>
     <row r="5">
@@ -547,16 +547,16 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>22249324.22</v>
+        <v>56774778.73</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2472147.14</v>
+        <v>2468468.64</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4.5</v>
+        <v>3.83</v>
       </c>
     </row>
   </sheetData>
@@ -619,13 +619,13 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>134</v>
+        <v>403</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>163410778.09</v>
+        <v>535380308.9</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>67</v>
+        <v>67.17</v>
       </c>
     </row>
     <row r="3">
@@ -640,13 +640,13 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46660689.06</v>
+        <v>115233866.05</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>13.5</v>
+        <v>14.67</v>
       </c>
     </row>
     <row r="4">
@@ -661,13 +661,13 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>18297501.12</v>
+        <v>47456454.08</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>8</v>
+        <v>6.17</v>
       </c>
     </row>
     <row r="5">
@@ -682,13 +682,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>23332363.45</v>
+        <v>72572038.73</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>7</v>
+        <v>8.17</v>
       </c>
     </row>
     <row r="6">
@@ -703,13 +703,13 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7692449.57</v>
+        <v>23900741.37</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>4.5</v>
+        <v>3.83</v>
       </c>
     </row>
   </sheetData>
@@ -726,7 +726,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -756,16 +756,16 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>37</v>
+        <v>32.62</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>19.01</v>
+        <v>18.11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>11.96</v>
+        <v>12.14</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2.97</v>
+        <v>3.01</v>
       </c>
     </row>
   </sheetData>
@@ -782,7 +782,7 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -836,56 +836,56 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Kaduna</t>
+          <t>Rivers</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>40498244.53</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F2" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="n">
-        <v>22231074.77</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="G2" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Oyo State Government</t>
+          <t>Lagos State Government</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Kano</t>
+          <t>Delta</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>38589896.35</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>19927339.63</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G3" s="3" t="n">
-        <v>0</v>
+        <v>38.46</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Nigerian Army</t>
+          <t>Kano State Government</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -894,208 +894,208 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>17415158.13</v>
+        <v>34212520.99</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>3.32</v>
+        <v>2.21</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0</v>
+        <v>18.18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>CBN</t>
+          <t>Nigerian Army</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Kano</t>
+          <t>Kaduna</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>17109775.57</v>
+        <v>33931065.65</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3.26</v>
+        <v>2.19</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Federal Ministry of Finance</t>
+          <t>NNPC</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Kaduna</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>33289037.02</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="3" t="n">
-        <v>13939385.41</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="G6" s="3" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Lagos State Government</t>
+          <t>NNPC</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Enugu</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>31684823.21</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="F7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="3" t="n">
-        <v>13755112.43</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="G7" s="3" t="n">
-        <v>50</v>
+        <v>28.57</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Federal Ministry of Finance</t>
+          <t>NNPC</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Enugu</t>
+          <t>Kano</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>13568918.25</v>
+        <v>30567259.86</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2.59</v>
+        <v>1.98</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>20</v>
+        <v>22.22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Oyo State Government</t>
+          <t>CBN</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Abuja</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>13313593.82</v>
+        <v>30484557.79</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2.54</v>
+        <v>1.97</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Oyo State Government</t>
+          <t>NNPC</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Kaduna</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>12301269.9</v>
+        <v>30083662.03</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2.35</v>
+        <v>1.94</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Rivers State Government</t>
+          <t>CBN</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Oyo</t>
+          <t>Kano</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>12143641.53</v>
+        <v>29622517.22</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2.32</v>
+        <v>1.91</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1173,187 +1173,187 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>NNPC</t>
+          <t>Oyo State Government</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>65988505.79</v>
+        <v>209275067.56</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>44635250.2</v>
+        <v>161452427.91</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>67.64</v>
+        <v>77.15000000000001</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>21353255.59</v>
+        <v>47822639.65</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>33</v>
+        <v>218</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>63</v>
+        <v>135</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>172</v>
+        <v>714</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Oyo State Government</t>
+          <t>Lagos State Government</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>90264244.44</v>
+        <v>197747036.64</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>63516379.93</v>
+        <v>152928033.81</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>70.37</v>
+        <v>77.34</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26747864.51</v>
+        <v>44819002.83</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>108</v>
+        <v>179</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>51</v>
+        <v>167</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>273</v>
+        <v>603</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Nigerian Police Force</t>
+          <t>CBN</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>56002385.22</v>
+        <v>197627199.33</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>40930629.75</v>
+        <v>155620230.17</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>73.09</v>
+        <v>78.73999999999999</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>15071755.47</v>
+        <v>42006969.16</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>40</v>
+        <v>93</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>25</v>
+        <v>115</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>157</v>
+        <v>563</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Lagos State Government</t>
+          <t>NNPC</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>63127266.78</v>
+        <v>270281379.92</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>48461733.98</v>
+        <v>217101345.17</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>76.77</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>14665532.8</v>
+        <v>53180034.75</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>68</v>
+        <v>178</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>185</v>
+        <v>853</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>CBN</t>
+          <t>Rivers State Government</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>73629978.03</v>
+        <v>160028037.31</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>57588092.39</v>
+        <v>129200075.14</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>78.20999999999999</v>
+        <v>80.73999999999999</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>16041885.64</v>
+        <v>30827962.17</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>217</v>
+        <v>555</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Federal Ministry of Finance</t>
+          <t>Nigerian Police Force</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>73007531.76000001</v>
+        <v>166466929.54</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>59529633.83</v>
+        <v>134762278.96</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>81.54000000000001</v>
+        <v>80.95</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>13477897.93</v>
+        <v>31704650.58</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>56</v>
+        <v>103</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>189</v>
+        <v>576</v>
       </c>
     </row>
     <row r="8">
@@ -1363,59 +1363,59 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>47563556.28</v>
+        <v>172604544.22</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>39408743</v>
+        <v>140727488.67</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>82.84999999999999</v>
+        <v>81.53</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>8154813.28</v>
+        <v>31877055.55</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>18</v>
+        <v>98</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>152</v>
+        <v>617</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Rivers State Government</t>
+          <t>Federal Ministry of Finance</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>67476159.5</v>
+        <v>184056837.11</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>56733777.16</v>
+        <v>150329650.35</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>84.08</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>10742382.34</v>
+        <v>33727186.76</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>39</v>
+        <v>108</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>31</v>
+        <v>122</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>252</v>
+        <v>603</v>
       </c>
     </row>
     <row r="10">
@@ -1425,28 +1425,28 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>58017626.1</v>
+        <v>185669033.06</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>49323183.41</v>
+        <v>153037587.55</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>85.01000000000001</v>
+        <v>82.42</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>8694442.689999999</v>
+        <v>32631445.51</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>24</v>
+        <v>112</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>38</v>
+        <v>135</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>190</v>
+        <v>647</v>
       </c>
     </row>
     <row r="11">
@@ -1456,28 +1456,28 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>67441736.81999999</v>
+        <v>210242658.78</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>62063786.02</v>
+        <v>179475893.86</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>92.03</v>
+        <v>85.37</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>5377950.8</v>
+        <v>30766764.92</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>28</v>
+        <v>106</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>35</v>
+        <v>121</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>309</v>
+        <v>799</v>
       </c>
     </row>
   </sheetData>

</xml_diff>